<commit_message>
Populate topics table with subtopics
</commit_message>
<xml_diff>
--- a/relatorio_subtopicos_erros.xlsx
+++ b/relatorio_subtopicos_erros.xlsx
@@ -397,10 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C71"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
     <col min="3" max="3" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -420,7 +420,7 @@
         <v>Esquistossomose</v>
       </c>
       <c r="B2" t="str">
-        <v>Esquistossomose Intestinal: Diagnóstico Histopatológico</v>
+        <v>Diagnostico histopatologico da esquistossomose (granulomas periovulares)</v>
       </c>
       <c r="C2" t="str">
         <v>84.6_x000d_</v>
@@ -431,7 +431,7 @@
         <v>Imunização</v>
       </c>
       <c r="B3" t="str">
-        <v>Vacinação Pneumocócica em Adultos com Comorbidades</v>
+        <v>Recomendacao de vacina pneumococica conjugada apos VPP23 (adulto com comorbidades)</v>
       </c>
       <c r="C3" t="str">
         <v>84.6_x000d_</v>
@@ -442,7 +442,7 @@
         <v>Hepatite C</v>
       </c>
       <c r="B4" t="str">
-        <v>Hepatite C: Tratamento com Antivirais de Ação Direta (DAA)</v>
+        <v>Esquema de primeira linha com DAA para hepatite C (genotipo 1)</v>
       </c>
       <c r="C4" t="str">
         <v>66.7_x000d_</v>
@@ -453,7 +453,7 @@
         <v>Imunização</v>
       </c>
       <c r="B5" t="str">
-        <v>Vacinas de Vírus Vivo em Pacientes Imunossuprimidos (Usuários de Imunobiológicos)</v>
+        <v>Contraindicacao de vacina de virus vivo em uso de infliximabe</v>
       </c>
       <c r="C5" t="str">
         <v>66.7_x000d_</v>
@@ -464,7 +464,7 @@
         <v>Tuberculose</v>
       </c>
       <c r="B6" t="str">
-        <v>Tuberculose Extrapulmonar: Meningoencefalite (Diagnóstico e Tratamento)</v>
+        <v>Diagnostico e tratamento da meningoencefalite tuberculosa</v>
       </c>
       <c r="C6" t="str">
         <v>66.7_x000d_</v>
@@ -475,7 +475,7 @@
         <v>Tuberculose</v>
       </c>
       <c r="B7" t="str">
-        <v>Tuberculose Multirresistente (TB-MDR): Diagnóstico e Manejo</v>
+        <v>Resistencia a rifampicina no TRM-TB: manejo da TB-MDR</v>
       </c>
       <c r="C7" t="str">
         <v>66.7_x000d_</v>
@@ -486,7 +486,7 @@
         <v>Hepatite B</v>
       </c>
       <c r="B8" t="str">
-        <v>Reativação do HBV em Pacientes Imunossuprimidos: Profilaxia</v>
+        <v>Profilaxia de reativacao do HBV antes de anti-TNF (Anti-HBc positivo)</v>
       </c>
       <c r="C8" t="str">
         <v>61.5_x000d_</v>
@@ -497,7 +497,7 @@
         <v>Tuberculose</v>
       </c>
       <c r="B9" t="str">
-        <v>Tuberculose: Falha Terapêutica e Resistência Medicamentosa</v>
+        <v>Falha terapeutica da TB: baciloscopia positiva apos 2 meses de RIPE</v>
       </c>
       <c r="C9" t="str">
         <v>61.5_x000d_</v>
@@ -508,7 +508,7 @@
         <v>Doenças Exantemáticas</v>
       </c>
       <c r="B10" t="str">
-        <v>Caxumba: Complicações em homens pós-púberes</v>
+        <v>Complicacoes da caxumba em homens pos-puberes</v>
       </c>
       <c r="C10" t="str">
         <v>58.3_x000d_</v>
@@ -519,7 +519,7 @@
         <v>Febre Amarela</v>
       </c>
       <c r="B11" t="str">
-        <v>Febre Amarela Urbana: Forma Grave e Diagnóstico</v>
+        <v>Forma grave de febre amarela: diagnostico clinico</v>
       </c>
       <c r="C11" t="str">
         <v>58.3_x000d_</v>
@@ -530,7 +530,7 @@
         <v>Infecções Oportunistas</v>
       </c>
       <c r="B12" t="str">
-        <v>Pneumonia por Pneumocystis jirovecii (PCP): Tratamento</v>
+        <v>Tratamento da pneumonia por Pneumocystis jirovecii (transplantado renal)</v>
       </c>
       <c r="C12" t="str">
         <v>58.3_x000d_</v>
@@ -541,7 +541,7 @@
         <v>Leishmaniose</v>
       </c>
       <c r="B13" t="str">
-        <v>Leishmaniose Visceral (Calazar): Diagnóstico Clínico</v>
+        <v>Diagnostico clinico do calazar (hepatoesplenomegalia e pancitopenia)</v>
       </c>
       <c r="C13" t="str">
         <v>58.3_x000d_</v>
@@ -549,21 +549,21 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Febre de Origem Indeterminada (FOI)</v>
+        <v>Tuberculose</v>
       </c>
       <c r="B14" t="str">
-        <v>Investigação Diagnóstica da FOI</v>
+        <v>Interpretacao do PPD em contato domiciliar com BCG (8 mm)</v>
       </c>
       <c r="C14" t="str">
-        <v>53.8_x000d_</v>
+        <v>58.3_x000d_</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Infecções Oportunistas</v>
+        <v>Febre de Origem Indeterminada (FOI)</v>
       </c>
       <c r="B15" t="str">
-        <v>Profilaxia Primária em Pacientes com HIV (Pneumocistose/Toxoplasmose)</v>
+        <v>Proximo passo na investigacao de febre de origem indeterminada</v>
       </c>
       <c r="C15" t="str">
         <v>53.8_x000d_</v>
@@ -571,10 +571,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Sepse e Choque Séptico</v>
+        <v>Infecções Oportunistas</v>
       </c>
       <c r="B16" t="str">
-        <v>Choque Séptico de Foco Urinário: Antibioticoterapia Empírica</v>
+        <v>Profilaxia primaria de infeccoes oportunistas em HIV (CD4 180)</v>
       </c>
       <c r="C16" t="str">
         <v>53.8_x000d_</v>
@@ -582,21 +582,21 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>Sepse e Choque Séptico</v>
       </c>
       <c r="B17" t="str">
-        <v>Mononucleose Infecciosa: Diagnóstico Diferencial</v>
+        <v>Antibioticoterapia empirica no choque septico de foco urinario</v>
       </c>
       <c r="C17" t="str">
-        <v>50.0_x000d_</v>
+        <v>53.8_x000d_</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Imunização</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B18" t="str">
-        <v>Vacina Tríplice Viral (MMR): Falsas Contraindicações (Alergia ao Ovo)</v>
+        <v>Diagnostico diferencial de mononucleose infecciosa</v>
       </c>
       <c r="C18" t="str">
         <v>50.0_x000d_</v>
@@ -604,10 +604,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Pneumonia</v>
+        <v>Imunização</v>
       </c>
       <c r="B19" t="str">
-        <v>Derrame Pleural Parapneumônico e Empiema: Diagnóstico e Manejo</v>
+        <v>Vacina triplice viral e alergia ao ovo (falsa contraindicacao)</v>
       </c>
       <c r="C19" t="str">
         <v>50.0_x000d_</v>
@@ -615,10 +615,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Tuberculose</v>
+        <v>Pneumonia</v>
       </c>
       <c r="B20" t="str">
-        <v>Tratamento da Tuberculose: Efeitos Adversos (Neurite Óptica por Etambutol)</v>
+        <v>Manejo de empiema pleural (derrame complicado: drenagem mandatoria)</v>
       </c>
       <c r="C20" t="str">
         <v>50.0_x000d_</v>
@@ -626,21 +626,21 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>Tuberculose</v>
       </c>
       <c r="B21" t="str">
-        <v>Rubéola: Diagnóstico Clínico e Sinais Característicos</v>
+        <v>Neurite optica por etambutol: suspensao imediata</v>
       </c>
       <c r="C21" t="str">
-        <v>46.2_x000d_</v>
+        <v>50.0_x000d_</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Doenças Imunopreveníveis</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B22" t="str">
-        <v>Profilaxia do Tétano Acidental pós-exposição</v>
+        <v>Diagnostico clinico da rubeola (linfadenopatia retroauricular)</v>
       </c>
       <c r="C22" t="str">
         <v>46.2_x000d_</v>
@@ -648,10 +648,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>HIV/AIDS</v>
+        <v>Doenças Imunopreveníveis</v>
       </c>
       <c r="B23" t="str">
-        <v>Prevenção da Transmissão Vertical do HIV: Profilaxia do Recém-nascido</v>
+        <v>Profilaxia antitetanica em ferimento corto-contuso (esquema desconhecido)</v>
       </c>
       <c r="C23" t="str">
         <v>46.2_x000d_</v>
@@ -659,10 +659,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Imunização</v>
+        <v>HIV/AIDS</v>
       </c>
       <c r="B24" t="str">
-        <v>Vacinação contra Febre Amarela em Pacientes com HIV</v>
+        <v>Profilaxia da transmissao vertical do HIV no recem-nascido (CV materna detectavel)</v>
       </c>
       <c r="C24" t="str">
         <v>46.2_x000d_</v>
@@ -670,21 +670,21 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Brucelose</v>
+        <v>Imunização</v>
       </c>
       <c r="B25" t="str">
-        <v>Brucelose: Diagnóstico Clínico e Epidemiologia</v>
+        <v>Vacinacao contra febre amarela em paciente com HIV (CD4 adequado)</v>
       </c>
       <c r="C25" t="str">
-        <v>41.7_x000d_</v>
+        <v>46.2_x000d_</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>HIV/AIDS</v>
+        <v>Brucelose</v>
       </c>
       <c r="B26" t="str">
-        <v>Neurotoxoplasmose: Diagnóstico e Tratamento Empírico</v>
+        <v>Diagnostico clinico em veterinario (zoonose ocupacional)</v>
       </c>
       <c r="C26" t="str">
         <v>41.7_x000d_</v>
@@ -692,10 +692,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Infecções de Pele e Partes Moles</v>
+        <v>HIV/AIDS</v>
       </c>
       <c r="B27" t="str">
-        <v>Impetigo não bolhoso: Diagnóstico e Tratamento</v>
+        <v>Diagnostico e tratamento empirico da neurotoxoplasmose (lesoes anelares)</v>
       </c>
       <c r="C27" t="str">
         <v>41.7_x000d_</v>
@@ -703,10 +703,10 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Infecções do Trato Urinário</v>
+        <v>Infecções de Pele e Partes Moles</v>
       </c>
       <c r="B28" t="str">
-        <v>Cistite Aguda Não Complicada em Mulheres</v>
+        <v>Diagnostico e tratamento do impetigo nao bolhoso (lesoes melicericas)</v>
       </c>
       <c r="C28" t="str">
         <v>41.7_x000d_</v>
@@ -714,10 +714,10 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>IST (Infecções Sexualmente Transmissíveis)</v>
+        <v>Infecções do Trato Urinário</v>
       </c>
       <c r="B29" t="str">
-        <v>Donovanose (Granuloma Inguinal): Diagnóstico Clínico</v>
+        <v>Tratamento empirico de cistite aguda nao complicada em mulher jovem</v>
       </c>
       <c r="C29" t="str">
         <v>41.7_x000d_</v>
@@ -725,21 +725,21 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>IST (Infecções Sexualmente Transmissíveis)</v>
       </c>
       <c r="B30" t="str">
-        <v>Eritema Infeccioso (Quinta Doença): Diagnóstico Clínico</v>
+        <v>Diagnostico clinico da donovanose (ulceras granulomatosas indolores)</v>
       </c>
       <c r="C30" t="str">
-        <v>38.5_x000d_</v>
+        <v>41.7_x000d_</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>HIV/AIDS</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B31" t="str">
-        <v>Infecção Aguda pelo HIV (Síndrome Retroviral Aguda): Diagnóstico</v>
+        <v>Identificacao do agente etiologico do eritema infeccioso (parvovirus B19)</v>
       </c>
       <c r="C31" t="str">
         <v>38.5_x000d_</v>
@@ -747,10 +747,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Imunização</v>
+        <v>HIV/AIDS</v>
       </c>
       <c r="B32" t="str">
-        <v>Eventos Adversos Pós-Vacinação (EAPV): Reações Locais Comuns</v>
+        <v>Diagnostico da sindrome retroviral aguda (teste negativo inicial)</v>
       </c>
       <c r="C32" t="str">
         <v>38.5_x000d_</v>
@@ -761,7 +761,7 @@
         <v>Imunização</v>
       </c>
       <c r="B33" t="str">
-        <v>Varicela: Profilaxia Pós-Exposição em Profissionais de Saúde</v>
+        <v>Manejo de eventos adversos pos-vacinacao (reacao local da pentavalente)</v>
       </c>
       <c r="C33" t="str">
         <v>38.5_x000d_</v>
@@ -769,10 +769,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Leptospirose</v>
+        <v>Imunização</v>
       </c>
       <c r="B34" t="str">
-        <v>Leptospirose: Forma Grave (Doença de Weil)</v>
+        <v>Profilaxia pos-exposicao a varicela em profissional de saude (IgG negativo)</v>
       </c>
       <c r="C34" t="str">
         <v>38.5_x000d_</v>
@@ -780,10 +780,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Malária</v>
+        <v>Leptospirose</v>
       </c>
       <c r="B35" t="str">
-        <v>Malária: Diagnóstico Clínico e Laboratorial</v>
+        <v>Doenca de Weil: forma grave da leptospirose (IRA e hemorragia)</v>
       </c>
       <c r="C35" t="str">
         <v>38.5_x000d_</v>
@@ -791,10 +791,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Raiva</v>
+        <v>Malária</v>
       </c>
       <c r="B36" t="str">
-        <v>Raiva: Profilaxia Pós-Exposição em Acidentes de Alto Risco</v>
+        <v>Diagnostico laboratorial da malaria (esquema de picos febris)</v>
       </c>
       <c r="C36" t="str">
         <v>38.5_x000d_</v>
@@ -802,21 +802,21 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Acidentes por Animais Peçonhentos</v>
+        <v>Raiva</v>
       </c>
       <c r="B37" t="str">
-        <v>Acidente Crotálico (Cascavel): Diagnóstico e Tratamento</v>
+        <v>Profilaxia da raiva apos mordida de cao de rua (animal nao observavel)</v>
       </c>
       <c r="C37" t="str">
-        <v>33.3_x000d_</v>
+        <v>38.5_x000d_</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Dengue</v>
+        <v>Acidentes por Animais Peçonhentos</v>
       </c>
       <c r="B38" t="str">
-        <v>Dengue: Interpretação Laboratorial e Manejo</v>
+        <v>Identificacao do genero da serpente e indicacao de soro anticrotalico</v>
       </c>
       <c r="C38" t="str">
         <v>33.3_x000d_</v>
@@ -824,10 +824,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>HIV/AIDS</v>
+        <v>Dengue</v>
       </c>
       <c r="B39" t="str">
-        <v>HIV: Falha Virológica e Investigação de Resistência</v>
+        <v>Interpretacao de plaquetopenia estavel e conduta ambulatorial</v>
       </c>
       <c r="C39" t="str">
         <v>33.3_x000d_</v>
@@ -835,10 +835,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Sífilis</v>
+        <v>HIV/AIDS</v>
       </c>
       <c r="B40" t="str">
-        <v>Interpretação do seguimento sorológico (VDRL)</v>
+        <v>Investigacao de falha virologica do HIV (genotipagem)</v>
       </c>
       <c r="C40" t="str">
         <v>33.3_x000d_</v>
@@ -846,10 +846,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Tuberculose</v>
+        <v>Sífilis</v>
       </c>
       <c r="B41" t="str">
-        <v>Infecção Latente por Tuberculose (ILTB): Diagnóstico e Tratamento em Profissionais de Saúde</v>
+        <v>Interpretacao do VDRL pos-tratamento (queda de titulo 1:32 para 1:8)</v>
       </c>
       <c r="C41" t="str">
         <v>33.3_x000d_</v>
@@ -860,7 +860,7 @@
         <v>Tuberculose</v>
       </c>
       <c r="B42" t="str">
-        <v>Tratamento da Tuberculose: Monitoramento e Suspeita de Falha Terapêutica</v>
+        <v>Baciloscopia positiva no 2o mes: suspeita de falha terapeutica</v>
       </c>
       <c r="C42" t="str">
         <v>33.3_x000d_</v>
@@ -871,7 +871,7 @@
         <v>Doenças Exantemáticas</v>
       </c>
       <c r="B43" t="str">
-        <v>Sarampo: Diagnóstico Clínico e Sinais Patognomônicos</v>
+        <v>Diagnostico clinico do sarampo e sinais de Koplik</v>
       </c>
       <c r="C43" t="str">
         <v>30.8_x000d_</v>
@@ -882,7 +882,7 @@
         <v>Endocardite Infecciosa</v>
       </c>
       <c r="B44" t="str">
-        <v>Endocardite por Staphylococcus aureus: Tratamento (MSSA)</v>
+        <v>Tratamento da endocardite por MSSA (oxacilina sensivel)</v>
       </c>
       <c r="C44" t="str">
         <v>30.8_x000d_</v>
@@ -893,7 +893,7 @@
         <v>Hepatite B</v>
       </c>
       <c r="B45" t="str">
-        <v>Hepatite B Aguda: Diagnóstico Sorológico</v>
+        <v>Interpretacao sorologica da hepatite B aguda</v>
       </c>
       <c r="C45" t="str">
         <v>30.8_x000d_</v>
@@ -904,7 +904,7 @@
         <v>Hepatites Virais</v>
       </c>
       <c r="B46" t="str">
-        <v>Profilaxia Pós-Exposição (PEP) para Hepatite B</v>
+        <v>Profilaxia pos-exposicao sexual para hepatite B (nao vacinado)</v>
       </c>
       <c r="C46" t="str">
         <v>30.8_x000d_</v>
@@ -915,7 +915,7 @@
         <v>HIV/AIDS</v>
       </c>
       <c r="B47" t="str">
-        <v>Terapia Antirretroviral: Manejo da Falha Terapêutica e Terapia de Resgate</v>
+        <v>PEP apos exposicao sexual anal desprotegida (parceiro status desconhecido)</v>
       </c>
       <c r="C47" t="str">
         <v>30.8_x000d_</v>
@@ -923,10 +923,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Imunização</v>
+        <v>HIV/AIDS</v>
       </c>
       <c r="B48" t="str">
-        <v>Calendário Vacinal: Manejo de Atrasos Vacinais na Infância</v>
+        <v>Terapia de resgate para HIV com resistencia extensa (genotipagem)</v>
       </c>
       <c r="C48" t="str">
         <v>30.8_x000d_</v>
@@ -934,10 +934,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Paracoccidioidomicose</v>
+        <v>Imunização</v>
       </c>
       <c r="B49" t="str">
-        <v>Paracoccidioidomicose: Forma Crônica e Diagnóstico Clínico</v>
+        <v>Manejo de atrasos vacinais na infancia (esquema catch-up)</v>
       </c>
       <c r="C49" t="str">
         <v>30.8_x000d_</v>
@@ -945,21 +945,21 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>Paracoccidioidomicose</v>
       </c>
       <c r="B50" t="str">
-        <v>Exantema Súbito (Roséola Infantil): Diagnóstico Clínico</v>
+        <v>Diagnostico da paracoccidioidomicose (padrao asa de borboleta e mucosa oral)</v>
       </c>
       <c r="C50" t="str">
-        <v>25.0_x000d_</v>
+        <v>30.8_x000d_</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Hanseníase</v>
+        <v>Coinfecção Tuberculose/HIV</v>
       </c>
       <c r="B51" t="str">
-        <v>Hanseníase Tuberculoide: Diagnóstico Clínico</v>
+        <v>SIRI em tuberculose pulmonar: diagnostico</v>
       </c>
       <c r="C51" t="str">
         <v>25.0_x000d_</v>
@@ -967,10 +967,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Tuberculose</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B52" t="str">
-        <v>Tratamento da Tuberculose: Efeitos Adversos (Hiperuricemia por Pirazinamida)</v>
+        <v>Diagnostico clinico da roseola infantil (HHV-6)</v>
       </c>
       <c r="C52" t="str">
         <v>25.0_x000d_</v>
@@ -978,10 +978,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Tuberculose</v>
+        <v>Hanseníase</v>
       </c>
       <c r="B53" t="str">
-        <v>Tuberculose: Efeitos Adversos do Tratamento (Hiperuricemia)</v>
+        <v>Diagnostico clinico da hanseniase tuberculoide (hipoestesia e espessamento neural)</v>
       </c>
       <c r="C53" t="str">
         <v>25.0_x000d_</v>
@@ -989,32 +989,32 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Coinfecção Tuberculose/HIV</v>
+        <v>Tuberculose</v>
       </c>
       <c r="B54" t="str">
-        <v>Interações Medicamentosas entre TARV e Tuberculostáticos (Dolutegravir e Rifampicina)</v>
+        <v>Hiperuricemia e artrite por pirazinamida: diagnostico e conduta</v>
       </c>
       <c r="C54" t="str">
-        <v>23.1_x000d_</v>
+        <v>25.0_x000d_</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Dengue</v>
+        <v>Tuberculose</v>
       </c>
       <c r="B55" t="str">
-        <v>Dengue: Classificação de Risco e Manejo (Sinais de Alarme)</v>
+        <v>Hiperuricemia por pirazinamida no tratamento da TB: identificacao do farmaco</v>
       </c>
       <c r="C55" t="str">
-        <v>23.1_x000d_</v>
+        <v>25.0_x000d_</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>Coinfecção Tuberculose/HIV</v>
       </c>
       <c r="B56" t="str">
-        <v>Escarlatina: Diagnóstico e Tratamento</v>
+        <v>Manejo da interacao Dolutegravir e Rifampicina</v>
       </c>
       <c r="C56" t="str">
         <v>23.1_x000d_</v>
@@ -1022,10 +1022,10 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Imunização</v>
+        <v>Dengue</v>
       </c>
       <c r="B57" t="str">
-        <v>Imunização do Viajante: Recomendações para o Sudeste Asiático</v>
+        <v>Classificacao de dengue com sinais de alarme e conduta imediata</v>
       </c>
       <c r="C57" t="str">
         <v>23.1_x000d_</v>
@@ -1033,10 +1033,10 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>Imunização</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B58" t="str">
-        <v>Vacinação na Gestação e Puerpério (Rubéola)</v>
+        <v>Diagnostico clinico e tratamento da escarlatina</v>
       </c>
       <c r="C58" t="str">
         <v>23.1_x000d_</v>
@@ -1044,10 +1044,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>Infecções Respiratórias Virais</v>
+        <v>Imunização</v>
       </c>
       <c r="B59" t="str">
-        <v>Influenza: Complicações (Pneumonia Bacteriana Secundária)</v>
+        <v>Manejo de suscetibilidade a rubeola na gestacao (vacinacao no puerperio)</v>
       </c>
       <c r="C59" t="str">
         <v>23.1_x000d_</v>
@@ -1055,24 +1055,24 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>Coinfecção Tuberculose/HIV</v>
+        <v>Imunização</v>
       </c>
       <c r="B60" t="str">
-        <v>Síndrome Inflamatória da Reconstituição Imune (SIRI)</v>
+        <v>Recomendacoes vacinais para viajante ao Sudeste Asiatico</v>
       </c>
       <c r="C60" t="str">
-        <v>20.0_x000d_</v>
+        <v>23.1_x000d_</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>HIV/AIDS</v>
+        <v>Infecções Respiratórias Virais</v>
       </c>
       <c r="B61" t="str">
-        <v>Profilaxia Pós-Exposição (PEP) ao HIV</v>
+        <v>Pneumonia bacteriana secundaria a influenza (piora apos melhora inicial)</v>
       </c>
       <c r="C61" t="str">
-        <v>19.2_x000d_</v>
+        <v>23.1_x000d_</v>
       </c>
     </row>
     <row r="62">
@@ -1080,7 +1080,7 @@
         <v>Doenças Diarreicas Agudas</v>
       </c>
       <c r="B62" t="str">
-        <v>Manejo inicial da gastroenterite aguda não complicada</v>
+        <v>Orientacao inicial em gastroenterite aguda sem desidratacao</v>
       </c>
       <c r="C62" t="str">
         <v>16.7_x000d_</v>
@@ -1091,7 +1091,7 @@
         <v>Ectoparasitoses</v>
       </c>
       <c r="B63" t="str">
-        <v>Escabiose: Diagnóstico e Manejo de Contatos</v>
+        <v>Diagnostico e manejo de contatos na escabiose</v>
       </c>
       <c r="C63" t="str">
         <v>16.7_x000d_</v>
@@ -1099,10 +1099,10 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Histoplasmose</v>
+        <v>Coinfecção Tuberculose/HIV</v>
       </c>
       <c r="B64" t="str">
-        <v>Histoplasmose Pulmonar Aguda: Diagnóstico e Epidemiologia</v>
+        <v>SIRI em neurotoxoplasmose: hipotese e conduta</v>
       </c>
       <c r="C64" t="str">
         <v>15.4_x000d_</v>
@@ -1110,21 +1110,21 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>Doenças Exantemáticas</v>
+        <v>Histoplasmose</v>
       </c>
       <c r="B65" t="str">
-        <v>Herpes Zoster: Diagnóstico e Prevenção de Neuralgia Pós-Herpética</v>
+        <v>Diagnostico e epidemiologia da histoplasmose (exposicao a galinheiro)</v>
       </c>
       <c r="C65" t="str">
-        <v>8.3_x000d_</v>
+        <v>15.4_x000d_</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>Infecções Intra-abdominais</v>
+        <v>Doenças Exantemáticas</v>
       </c>
       <c r="B66" t="str">
-        <v>Colangite Aguda: Diagnóstico e Tratamento</v>
+        <v>Diagnostico e prevencao de neuralgia pos-herpetica</v>
       </c>
       <c r="C66" t="str">
         <v>8.3_x000d_</v>
@@ -1132,10 +1132,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>Infecções Oportunistas</v>
+        <v>Infecções Intra-abdominais</v>
       </c>
       <c r="B67" t="str">
-        <v>Neurocriptococose: Diagnóstico e Tratamento</v>
+        <v>Diagnostico e conduta inicial da colangite aguda (triade de Charcot)</v>
       </c>
       <c r="C67" t="str">
         <v>8.3_x000d_</v>
@@ -1143,18 +1143,51 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>Tuberculose</v>
+        <v>Infecções Oportunistas</v>
       </c>
       <c r="B68" t="str">
-        <v>Tratamento da Tuberculose: Interações Medicamentosas (Rifampicina e Contraceptivos)</v>
+        <v>Diagnostico e tratamento da neurocriptococose (tinta da China positiva)</v>
       </c>
       <c r="C68" t="str">
         <v>8.3_x000d_</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Tuberculose</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Interacao rifampicina e anticoncepcional oral: orientacao contraceptiva</v>
+      </c>
+      <c r="C69" t="str">
+        <v>8.3_x000d_</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Tuberculose</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Interpretacao do PPD em profissional de saude (12 mm, sem BCG)</v>
+      </c>
+      <c r="C70" t="str">
+        <v>8.3_x000d_</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>HIV/AIDS</v>
+      </c>
+      <c r="B71" t="str">
+        <v>PEP apos acidente percutaneo de alto risco (agulha contaminada)</v>
+      </c>
+      <c r="C71" t="str">
+        <v>7.7_x000d_</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C68"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C71"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>